<commit_message>
Update screenshots and modify CSRF tokens in HTML files
- Updated CSRF tokens in row9_activity_nature_error.html and row9_start_month_error.html to enhance security.
- Adjusted various HTML elements in row9_activity_nature_error.html for improved functionality and user experience.
- Updated multiple screenshot files to reflect recent changes in the application.
- Enhanced the result_writer.py script to normalize cell values and preserve bot status columns when generating output from existing workbooks.
</commit_message>
<xml_diff>
--- a/data/output.xlsx
+++ b/data/output.xlsx
@@ -61,12 +61,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00ED7D31"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ED7D31"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -107,10 +107,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -122,7 +119,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -632,97 +629,97 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 8 - Village with Good Governance</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Activities realted to Record keeping /Maintainance of data base</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Maintenance of community system</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 1</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-100</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Women,Youth</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>July</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>100</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>20</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>10</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>50000</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
@@ -732,7 +729,7 @@
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>2026-06-29 16:37:26</t>
+          <t>2026-06-29 17:41:19</t>
         </is>
       </c>
       <c r="V2" s="3" t="inlineStr"/>
@@ -740,97 +737,97 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 5 - Clean and Green Village</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Awareness generation for use of natural products in daily life</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Social forestry and farm forestry</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 2</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-101</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>August</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>110</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>11</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>60000</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
@@ -840,7 +837,7 @@
       </c>
       <c r="U3" s="3" t="inlineStr">
         <is>
-          <t>2026-06-29 16:37:30</t>
+          <t>2026-06-29 17:41:25</t>
         </is>
       </c>
       <c r="V3" s="3" t="inlineStr"/>
@@ -848,97 +845,97 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 2 - Healthy Village</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Awareness camp on behavioural issues of Mission LiFE</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Beneficiary Oriented Programmes</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 3</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Whether Training for Disaster Management conducted</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Women,Youth</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>September</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>120</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>24</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>12</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>70000</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
@@ -948,7 +945,7 @@
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-29 16:37:35</t>
+          <t>2026-06-29 17:41:30</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr"/>
@@ -956,209 +953,205 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 8 - Village with Good Governance</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Awareness campaign on SHG-PRI Convergence</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Social welfare</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Beneficiary Oriented Programmes</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 4</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-103</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>October</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>130</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>26</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>13</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="T5" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U5" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:37:56</t>
-        </is>
-      </c>
-      <c r="V5" s="4" t="inlineStr">
-        <is>
-          <t>[activity_nature] 'Maintenance' not found in #workTypId. Available (1): ['New/Fresh']</t>
-        </is>
-      </c>
+          <t>80000</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:41:36</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 4 - Water Sufficient Village</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Amrit Sarovar/Pond/Farm Pond</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Drinking water</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 5</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-104</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Women,Youth</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>November</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>140</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>28</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>14</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>90000</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
@@ -1168,7 +1161,7 @@
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>2026-06-29 16:38:02</t>
+          <t>2026-06-29 17:41:41</t>
         </is>
       </c>
       <c r="V6" s="3" t="inlineStr"/>
@@ -1176,97 +1169,97 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 8 - Village with Good Governance</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Awareness for active participation in Gram Sabha, Ward Sabha, Mahila Sabha</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Social welfare</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 6</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-105</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>6</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>December</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>150</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>30</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>100000</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
@@ -1276,7 +1269,7 @@
       </c>
       <c r="U7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-29 16:38:08</t>
+          <t>2026-06-29 17:41:46</t>
         </is>
       </c>
       <c r="V7" s="3" t="inlineStr"/>
@@ -1284,1010 +1277,974 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 7 - Socially Just and Socially Secured Village</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Awareness Campaign  pension</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Welfare of the weaker sections</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 7</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-106</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Women,Youth</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>April</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>160</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>32</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>16</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="T8" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:38:28</t>
-        </is>
-      </c>
-      <c r="V8" s="4" t="inlineStr">
-        <is>
-          <t>[activity_nature] 'Maintenance' not found in #workTypId. Available (1): ['New/Fresh'] | [start_month] 'January' not found in #startMonthId. Available (9): ['April', 'May', 'June', 'July', 'August', 'September', 'October', 'November', 'December']</t>
-        </is>
-      </c>
+          <t>110000</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:41:51</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 8 - Village with Good Governance</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Awareness on Public Services/ Service Delivery Provisions/ RTI</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Social welfare</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 8</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-107</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>April</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>170</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>34</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>17</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="T9" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U9" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:38:49</t>
-        </is>
-      </c>
-      <c r="V9" s="4" t="inlineStr">
-        <is>
-          <t>[start_month] 'February' not found in #startMonthId. Available (9): ['April', 'May', 'June', 'July', 'August', 'September', 'October', 'November', 'December']</t>
-        </is>
-      </c>
+          <t>120000</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:41:57</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 6 - Self-sufficient Infrastructure in Village</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Annual Expenses - Water Charges, Postal, Electricity Bills, Internet Bill, Printing Charges</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Maintenance of community system</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 9</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-108</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Women,Youth</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>March</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>180</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>36</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>18</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="T10" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U10" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:39:08</t>
-        </is>
-      </c>
-      <c r="V10" s="4" t="inlineStr">
-        <is>
-          <t>[activity_nature] 'New/Fresh' not found in #workTypId. Available (1): ['Operational']</t>
-        </is>
-      </c>
+          <t>130000</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:42:02</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 8 - Village with Good Governance</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Awareness on disaster preparedness and mitigation</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Poverty allevation programme</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 10</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-109</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>January</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>190</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>38</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>19</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="T11" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U11" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:39:31</t>
-        </is>
-      </c>
-      <c r="V11" s="4" t="inlineStr">
-        <is>
-          <t>[activity_nature] 'Maintenance' not found in #workTypId. Available (1): ['New/Fresh'] | [start_month] 'April' not found in #startMonthId. Available (3): ['January', 'February', 'March']</t>
-        </is>
-      </c>
+          <t>140000</t>
+        </is>
+      </c>
+      <c r="T11" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="U11" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:42:08</t>
+        </is>
+      </c>
+      <c r="V11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 8 - Village with Good Governance</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Awareness on inclusion of beneficiaries under different scheme</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Social welfare</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 11</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-110</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Women,Youth</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>January</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>200</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>40</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>20</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="T12" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U12" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:39:54</t>
-        </is>
-      </c>
-      <c r="V12" s="4" t="inlineStr">
-        <is>
-          <t>[start_month] 'May' not found in #startMonthId. Available (3): ['January', 'February', 'March']</t>
-        </is>
-      </c>
+          <t>150000</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:42:15</t>
+        </is>
+      </c>
+      <c r="V12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 3 - Child Friendly Village</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Awareness Campaign on services of ICDS</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Women and child development</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 12</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-111</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>6</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>January</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>210</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>42</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>21</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="T13" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U13" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:40:21</t>
-        </is>
-      </c>
-      <c r="V13" s="4" t="inlineStr">
-        <is>
-          <t>[start_month] 'June' not found in #startMonthId. Available (3): ['January', 'February', 'March']</t>
-        </is>
-      </c>
+          <t>160000</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:42:20</t>
+        </is>
+      </c>
+      <c r="V13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 8 - Village with Good Governance</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Capacity Building &amp; Training of Elected Representatives &amp; Functionaries</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Social welfare</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 13</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-112</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Women,Youth</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>January</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>220</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>44</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>22</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="T14" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U14" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:40:44</t>
-        </is>
-      </c>
-      <c r="V14" s="4" t="inlineStr">
-        <is>
-          <t>[activity_nature] 'Maintenance' not found in #workTypId. Available (1): ['New/Fresh'] | [start_month] 'July' not found in #startMonthId. Available (3): ['January', 'February', 'March']</t>
-        </is>
-      </c>
+          <t>170000</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:42:26</t>
+        </is>
+      </c>
+      <c r="V14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 9 - Women Friendly Village</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Access to Maternal Benefits</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Women and child development</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 14</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-113</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>January</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>230</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>46</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>23</t>
         </is>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="T15" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U15" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:41:07</t>
-        </is>
-      </c>
-      <c r="V15" s="4" t="inlineStr">
-        <is>
-          <t>[start_month] 'August' not found in #startMonthId. Available (3): ['January', 'February', 'March']</t>
-        </is>
-      </c>
+          <t>180000</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:42:32</t>
+        </is>
+      </c>
+      <c r="V15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Theme 8 - Village with Good Governance</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Charages / Fees and other activites for ISO Certification</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>GP Office Infrastructure</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Sample activity description for record 15</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PDI-114</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>All</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Women,Youth</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>January</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>240</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>48</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>24</t>
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="T16" s="4" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U16" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:41:30</t>
-        </is>
-      </c>
-      <c r="V16" s="4" t="inlineStr">
-        <is>
-          <t>[start_month] 'September' not found in #startMonthId. Available (3): ['January', 'February', 'March']</t>
-        </is>
-      </c>
+          <t>190000</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:42:40</t>
+        </is>
+      </c>
+      <c r="V16" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2308,86 +2265,86 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Total Records</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Successful</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>5</t>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Success Rate</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>33.3%</t>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Execution Time (s)</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>643.1</t>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>164.6</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Completed At</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>2026-06-29 16:41:30</t>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:42:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Enhance activity output handling and migration process
- Updated `run` function in `main.py` to include output repository parameter.
- Modified retry mechanism to use `page.wait_for_timeout` for better handling.
- Refactored `ResultWriter` in `result_writer.py` to support dynamic sheet name resolution and improved header normalization.
- Introduced `workbook_migration.py` for migrating legacy activity sheets to a new format, including validation and error handling.
- Added unit tests in `test_activity_output_architecture.py` to ensure proper functionality of activity key normalization, output type handling, and training validation.
- Implemented checks for duplicate and missing activity keys in the workbook migration process.
</commit_message>
<xml_diff>
--- a/data/output.xlsx
+++ b/data/output.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="eGram Activity Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Activities" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Automation_Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -56,7 +56,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -66,7 +66,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -116,10 +116,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -487,140 +487,218 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="60" customWidth="1" min="22" max="22"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
+    <col width="35" customWidth="1" min="23" max="23"/>
+    <col width="24" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="24" customWidth="1" min="27" max="27"/>
+    <col width="24" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="30" customWidth="1" min="30" max="30"/>
+    <col width="22" customWidth="1" min="31" max="31"/>
+    <col width="18" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="20" customWidth="1" min="34" max="34"/>
+    <col width="60" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>activity_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>theme</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>activity_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>focus_area</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>activity_type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>activity_description</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>pdi_indicator</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>activity_for</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>targeted_populace</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>activity_nature</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>is_directly_funded_by_panchayat</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>estimated_completion_year</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>estimated_completion_month</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>estimated_completion_days</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>start_year</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>start_month</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>expected_beneficiary_general</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>expected_beneficiary_sc</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>expected_beneficiary_st</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>indicative_unit_cost</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>total_indicative_cost</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>expected_results</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>flagship_scheme</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>select_supported_department</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>estimated_total_cost</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>shareable</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>major_head_choice</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>minor_head_choice</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>operation_type</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>operation_remarks</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>activity_output_type</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>final_action</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>processed_time</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>error_message</t>
         </is>
@@ -629,114 +707,155 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Theme 6 - Self-sufficient Infrastructure in Village</t>
+          <t>ACT-0001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Annual Expenses - Water Charges, Postal, Electricity Bills, Internet Bill, Printing Charges</t>
+          <t>Theme 2 - Healthy Village</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Maintenance of community system</t>
+          <t>Awareness camp on behavioural issues of Mission LiFE</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Community Works</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sample activity description for record 9</t>
+          <t>Beneficiary Oriented Programmes</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>PDI-108</t>
+          <t>Awareness camp on behavioural issues of Mission LiFE</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>Neonatal mortality rate (per 1,000 live births)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>All</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Women,Youth</t>
-        </is>
-      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>All</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>New/Fresh</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>March</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>180</t>
-        </is>
-      </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>10</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>10</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>Okay</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>ARI Division Schemes: Coir Udyami Yojana - Center Scheme</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>Department of Food &amp; Public Distribution</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
           <t>130000</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-30 18:20:47</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>[validation] Please check atlest one Mission Antyodyaya(MA) Gap(s)</t>
-        </is>
-      </c>
+      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AA2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>Training/Capacity Building</t>
+        </is>
+      </c>
+      <c r="AF2" s="2" t="inlineStr">
+        <is>
+          <t>Save and Forward</t>
+        </is>
+      </c>
+      <c r="AG2" s="3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="AH2" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07 17:03:10</t>
+        </is>
+      </c>
+      <c r="AI2" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -788,7 +907,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -800,7 +919,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -812,7 +931,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -824,7 +943,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>317.4</t>
+          <t>87.3</t>
         </is>
       </c>
     </row>
@@ -836,7 +955,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30 18:20:48</t>
+          <t>2026-07-07 17:03:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove obsolete screenshots and unused code; refactor output handling
- Deleted multiple error screenshot files that are no longer needed.
- Removed unused constants and functions from activity output handlers and registry.
- Refactored modal opening method in TrainingOutputHandler to simplify parameters.
- Cleaned up legacy code in form filler and result writer modules.
- Updated main execution flow to eliminate unnecessary variable assignments.
</commit_message>
<xml_diff>
--- a/data/output.xlsx
+++ b/data/output.xlsx
@@ -852,7 +852,7 @@
       </c>
       <c r="AH2" s="3" t="inlineStr">
         <is>
-          <t>2026-07-07 17:03:10</t>
+          <t>2026-07-07 17:42:29</t>
         </is>
       </c>
       <c r="AI2" s="3" t="inlineStr"/>
@@ -943,7 +943,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>87.3</t>
+          <t>80.0</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-07 17:03:10</t>
+          <t>2026-07-07 17:42:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add vprp_plan field to excel reader and form filler
- Introduced vprp_plan field in the FORM_COLUMNS of excel_reader.py.
- Enhanced ExcelReader class to handle shared output records for training activities.
- Implemented fill_vprp_plan function in form_filler.py to manage VPRP Plan radio button selection.
- Updated result_writer.py to include vprp_plan in the output columns.
- Modified workbook_migration.py to ensure vprp_plan is included in activity headers.
- Added tests for shared training records and PDI selection rules in test_activity_output_architecture.py.
</commit_message>
<xml_diff>
--- a/data/output.xlsx
+++ b/data/output.xlsx
@@ -56,7 +56,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -66,7 +66,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -116,10 +116,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI2"/>
+  <dimension ref="A1:AJ3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -496,35 +496,36 @@
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
     <col width="9" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="40" customWidth="1" min="22" max="22"/>
-    <col width="35" customWidth="1" min="23" max="23"/>
-    <col width="24" customWidth="1" min="24" max="24"/>
-    <col width="16" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="24" customWidth="1" min="27" max="27"/>
+    <col width="9" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="40" customWidth="1" min="23" max="23"/>
+    <col width="35" customWidth="1" min="24" max="24"/>
+    <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
     <col width="24" customWidth="1" min="28" max="28"/>
-    <col width="18" customWidth="1" min="29" max="29"/>
-    <col width="30" customWidth="1" min="30" max="30"/>
-    <col width="22" customWidth="1" min="31" max="31"/>
-    <col width="18" customWidth="1" min="32" max="32"/>
-    <col width="12" customWidth="1" min="33" max="33"/>
-    <col width="20" customWidth="1" min="34" max="34"/>
-    <col width="60" customWidth="1" min="35" max="35"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="30" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
+    <col width="18" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="20" customWidth="1" min="35" max="35"/>
+    <col width="60" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -560,145 +561,150 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>vprp_plan</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>pdi_indicator</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>activity_for</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>targeted_populace</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>activity_nature</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>is_directly_funded_by_panchayat</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>estimated_completion_year</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>estimated_completion_month</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>estimated_completion_days</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>start_year</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>start_month</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>expected_beneficiary_general</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>expected_beneficiary_sc</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>expected_beneficiary_st</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>indicative_unit_cost</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>total_indicative_cost</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>expected_results</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>flagship_scheme</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>select_supported_department</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>estimated_total_cost</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>shareable</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>major_head_choice</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>minor_head_choice</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>operation_type</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>operation_remarks</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>activity_output_type</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>final_action</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>processed_time</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>error_message</t>
         </is>
@@ -707,155 +713,302 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ACT-0001</t>
+          <t>ACT-0070</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Theme 2 - Healthy Village</t>
+          <t>Theme 3 - Child Friendly Village</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Awareness camp on behavioural issues of Mission LiFE</t>
+          <t>Child Participation, Leadership Strengthening &amp; Facilitation</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Beneficiary Oriented Programmes</t>
+          <t>Community Works</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Awareness camp on behavioural issues of Mission LiFE</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Neonatal mortality rate (per 1,000 live births)</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+          <t>Child Participation, Leadership Strengthening &amp; Facilitation</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>New/Fresh</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>March</t>
-        </is>
-      </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>April</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>8</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Okay</t>
+          <t>192</t>
         </is>
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>ARI Division Schemes: Coir Udyami Yojana - Center Scheme</t>
+          <t>Child Participation, Leadership Strengthening &amp; Facilitation</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>Department of Food &amp; Public Distribution</t>
-        </is>
-      </c>
-      <c r="Y2" s="2" t="inlineStr">
-        <is>
-          <t>130000</t>
-        </is>
-      </c>
+          <t>Pradhan Mantri Krishi Sinchayee Yojana (PMKSY) - Center Scheme</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr"/>
       <c r="Z2" s="2" t="inlineStr"/>
       <c r="AA2" s="2" t="inlineStr"/>
       <c r="AB2" s="2" t="inlineStr"/>
-      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>Whether the activity is for Elementary/Primary Education</t>
+        </is>
+      </c>
       <c r="AD2" s="2" t="inlineStr"/>
-      <c r="AE2" s="2" t="inlineStr">
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr">
         <is>
           <t>Training/Capacity Building</t>
         </is>
       </c>
-      <c r="AF2" s="2" t="inlineStr">
+      <c r="AG2" s="2" t="inlineStr">
         <is>
           <t>Save and Forward</t>
         </is>
       </c>
-      <c r="AG2" s="3" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
       <c r="AH2" s="3" t="inlineStr">
         <is>
-          <t>2026-07-09 12:13:30</t>
-        </is>
-      </c>
-      <c r="AI2" s="3" t="inlineStr"/>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="AI2" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-28 00:59:58</t>
+        </is>
+      </c>
+      <c r="AJ2" s="3" t="inlineStr">
+        <is>
+          <t>[activity_output] Training modal did not open: showTrainingDetailsPopup; diagnostics={'modalExists': True, 'modalClass': 'modal fade', 'modalDisplay': 'none', 'modalVisibility': 'visible', 'modalAriaHidden': None, 'radioExists': True, 'radioChecked': True, 'radioDisabled': False, 'radioOnclick': "return showAssetDetailsPopup('addassetdtlsDiv102',this.id);", 'outputTypeHidden': '', 'startMonthValue': '4', 'totalIndicativeCostValue': '192', 'totalExpectedBeneficiariesValue': '24', 'trainingCategoryVisible': False, 'hasModalBackdrop': False, 'visibleErrors': []}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ACT-0081</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Theme 3 - Child Friendly Village</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Institutional Strengthening &amp; Convergence on child related issues</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Women and child development</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Community Works</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Institutional Strengthening &amp; Convergence on child related issues</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>New/Fresh</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>Institutional Strengthening &amp; Convergence on child related issues</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>National Health Mission (NHM) - Center Scheme</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>Whether the activity is for Elementary/Primary Education</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>Training/Capacity Building</t>
+        </is>
+      </c>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>Save and Forward</t>
+        </is>
+      </c>
+      <c r="AH3" s="3" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="AI3" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-28 01:00:35</t>
+        </is>
+      </c>
+      <c r="AJ3" s="3" t="inlineStr">
+        <is>
+          <t>[activity_output] Training modal did not open: showTrainingDetailsPopup; diagnostics={'modalExists': True, 'modalClass': 'modal fade', 'modalDisplay': 'none', 'modalVisibility': 'visible', 'modalAriaHidden': None, 'radioExists': True, 'radioChecked': True, 'radioDisabled': False, 'radioOnclick': "return showAssetDetailsPopup('addassetdtlsDiv102',this.id);", 'outputTypeHidden': '', 'startMonthValue': '4', 'totalIndicativeCostValue': '80', 'totalExpectedBeneficiariesValue': '10', 'trainingCategoryVisible': False, 'hasModalBackdrop': False, 'visibleErrors': []}</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -895,7 +1048,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -907,7 +1060,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -919,7 +1072,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -931,7 +1084,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
@@ -943,7 +1096,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>84.2</t>
+          <t>165.9</t>
         </is>
       </c>
     </row>
@@ -955,7 +1108,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-07-09 12:13:31</t>
+          <t>2026-08-28 01:00:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance AssetOutputHandler with total units logging and callback tracing
- Added logging for total units value and type during processing.
- Implemented tracing for asset subcategory callbacks to ensure proper handling of total units.
- Enhanced logging around total units at various stages of the asset handling process.
- Improved error handling for coverage area selection and unit input persistence.
- Refactored input handling for total units and units per village to ensure accurate data entry.
</commit_message>
<xml_diff>
--- a/data/output.xlsx
+++ b/data/output.xlsx
@@ -851,24 +851,12 @@
       </c>
       <c r="AI2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-30 22:52:21</t>
+          <t>2026-08-30 23:19:50</t>
         </is>
       </c>
       <c r="AJ2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">[activity_output] Locator.check: Clicking the checkbox did not change its state
-Call log:
-  - waiting for locator("input#assetCovgeAreaId, input[name='assetDetails.astCvrgCd'][value='A']").first
-    - locator resolved to &lt;input value="A" type="radio" id="assetCovgeAreaId" name="assetDetails.astCvrgCd" onclick="showVillageForGPList(this.value)"/&gt;
-  - attempting click action
-    - scrolling into view if needed
-    - done scrolling
-    - forcing action
-    - performing click action
-    - click action done
-    - waiting for scheduled navigations to finish
-    - navigations have finished
-</t>
+          <t>[activity_output] Page.wait_for_function() takes 2 positional arguments but 3 positional arguments (and 1 keyword-only argument) were given</t>
         </is>
       </c>
     </row>
@@ -958,7 +946,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>12.3</t>
         </is>
       </c>
     </row>
@@ -970,7 +958,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-30 22:52:21</t>
+          <t>2026-08-30 23:19:50</t>
         </is>
       </c>
     </row>

</xml_diff>